<commit_message>
Final verification: genuine SAPI TTS + CC-BY footage run, verified MP4 output, honest audit of components, and updated submission workbook
</commit_message>
<xml_diff>
--- a/Assessment3_Abirami_Kumar.xlsx
+++ b/Assessment3_Abirami_Kumar.xlsx
@@ -851,7 +851,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>http://localhost:8000 (Docker Compose environment)</t>
+          <t>Not deployed to public cloud domain; runs locally via FastAPI at http://localhost:8000</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
       </c>
       <c r="B10" s="24" t="inlineStr">
         <is>
-          <t>None required (local / internal network deployment)</t>
+          <t>None required (local environment)</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       </c>
       <c r="B11" s="24" t="inlineStr">
         <is>
-          <t>0s (instant local container startup)</t>
+          <t>N/A (local environment)</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="B13" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/abiramikumar08/assess-3#demo-video (artifacts in test_pack/)</t>
+          <t>outputs/genuine_demo_run/video_16x9.mp4 (real 7.29s video with real SAPI narration &amp; real CC-BY footage)</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="B15" s="24" t="inlineStr">
         <is>
-          <t>Intel Core i7-12700H (16 vCPUs), 32 GB RAM, Windows 11 &amp; Docker Linux</t>
+          <t>Intel Core i7-12700H (16 vCPUs), 32 GB RAM, Windows 11 (Docker daemon not installed on host)</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>Supports plain script text, audio URL (WAV/MP3), or structured scenes list. Max 10 minutes (600s).</t>
+          <t>Text input generates real narration via Windows SAPI. Audio URLs accepted and duration extracted via ffprobe/wave, but automated Whisper speech-to-text transcription is not bundled; audio-only inputs use duration timestamps without word transcripts.</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>Pexels Free Commercial Licence + Synthetic mock assets. Source, licence, attribution, and AI flag in timeline.json.</t>
+          <t>Pexels Free Commercial Licence + Wikimedia Commons CC-BY clips + Synthetic mock assets. Source, licence, attribution, and AI flag in timeline.json.</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="D9" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/app/renderer.py:160-235 ; tests/test_pipeline.py::test_end_to_end_pipeline ; test_pack/01_finance_tutorial</t>
+          <t>ps3_engine/app/renderer.py:160-235 ; outputs/genuine_demo_run/video_16x9.mp4 ; tests/test_pipeline.py::test_end_to_end_pipeline</t>
         </is>
       </c>
       <c r="E9" s="24" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D13" s="24" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="E13" s="24" t="inlineStr">
         <is>
-          <t>All 10 Integration Standard points implemented and verified.</t>
+          <t>Integration Standard points 1-10 implemented in codebase; local Docker daemon was not installed so Compose startup was unverified locally, and no external public domain was hosted.</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/tests/test_pipeline.py (29 passed)</t>
+          <t>ps3_engine/tests/test_pipeline.py (30 passed)</t>
         </is>
       </c>
       <c r="E5" s="24" t="inlineStr">
@@ -1428,12 +1428,12 @@
       </c>
       <c r="D7" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/REPORT.md Section 4 ; test_pack/batch_summary.json</t>
+          <t>ps3_engine/REPORT.md Section 3 ; test_pack/batch_summary.json</t>
         </is>
       </c>
       <c r="E7" s="24" t="inlineStr">
         <is>
-          <t>Average measured relevance 4.2 / 5.0 across all 10 test video packs</t>
+          <t>Average measured relevance 4.2 / 5.0 across all 10 test video packs; 4.65 on genuine demo run</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>Pexels API commercial stock + Procedural mock video generator with fallback rule</t>
+          <t>Pexels API commercial stock + Wikimedia Commons CC-BY + Procedural mock video generator with fallback rule</t>
         </is>
       </c>
     </row>
@@ -1558,17 +1558,17 @@
       </c>
       <c r="C12" s="24" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/REPORT.md Section 4 &amp; 6</t>
+          <t>ps3_engine/REPORT.md Section 1</t>
         </is>
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
-          <t>Relevance scored per scene in timeline.json; independent VLM framework outlined</t>
+          <t>Automated VLM scoring not integrated; human heuristic rating used</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D13" s="24" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="E13" s="24" t="inlineStr">
         <is>
-          <t>Configurable TTS_LANGUAGE and phonetic duration modeling for multilingual voiceover</t>
+          <t>Configurable TTS_LANGUAGE and phonetic duration modeling; tested primarily on English voiceover</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/REPORT.md Section 4 &amp; 5</t>
+          <t>ps3_engine/REPORT.md Section 3</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Detailed turnaround, compute memory (145MB), cost (&lt;$0.002/min) and capacity metrics</t>
+          <t>Detailed turnaround, compute memory (120MB), cost ($0.00/min) and capacity metrics</t>
         </is>
       </c>
     </row>
@@ -1639,17 +1639,17 @@
       </c>
       <c r="C15" s="24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D15" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/REPORT.md Section 4 ; test_pack/batch_summary.json</t>
+          <t>ps3_engine/REPORT.md Section 3 ; test_pack/batch_summary.json</t>
         </is>
       </c>
       <c r="E15" s="24" t="inlineStr">
         <is>
-          <t>Curated semantic scene queries yield &gt;85% 4+ ratings in benchmark runs</t>
+          <t>Internal semantic scene rating achieves 4.2 average; formal external reviewer scoring pending</t>
         </is>
       </c>
     </row>
@@ -1764,12 +1764,12 @@
       </c>
       <c r="C5" s="24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/docker-compose.yml ; ps3_engine/.env.example ; pytest tests/</t>
+          <t>ps3_engine/docker-compose.yml ; ps3_engine/.env.example ; pytest tests/ (30 passed); local docker daemon not installed</t>
         </is>
       </c>
     </row>
@@ -1896,12 +1896,12 @@
       </c>
       <c r="C11" s="24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D11" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/app/api.py ; ps3_engine/app/renderer.py ; outputs/{job_id}/</t>
+          <t>ps3_engine/app/api.py ; ps3_engine/app/renderer.py ; outputs/{job_id}/ (local filesystem storage; live S3 bucket unconfigured)</t>
         </is>
       </c>
     </row>
@@ -2077,17 +2077,17 @@
       </c>
       <c r="C5" s="24" t="inlineStr">
         <is>
-          <t>12.4s (cold) / 8.1s (warm)</t>
+          <t>5.14s (genuine SAPI run) / 2.1s (mock)</t>
         </is>
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
-          <t>Intel Core i7-12700H, 16 vCPUs, 32GB RAM; 10 benchmark runs</t>
+          <t>Intel Core i7-12700H, 16 vCPUs, 32GB RAM; measured genuine pipeline execution</t>
         </is>
       </c>
       <c r="E5" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/REPORT.md Section 4 ; test_pack/batch_summary.json</t>
+          <t>ps3_engine/REPORT.md Section 3 ; outputs/genuine_demo_run/</t>
         </is>
       </c>
     </row>
@@ -2104,17 +2104,17 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>&lt; $0.002 / min</t>
+          <t>$0.00 / min</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>Pexels Free Commercial Licence + CPU encoding</t>
+          <t>Windows SAPI Speech + Open CC Wikimedia media; zero paid APIs used</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/REPORT.md Section 5</t>
+          <t>ps3_engine/REPORT.md Section 3</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="E7" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/app/renderer.py:200-225 ; outputs/*/timeline.json</t>
+          <t>ps3_engine/outputs/genuine_demo_run/timeline.json</t>
         </is>
       </c>
     </row>
@@ -2158,17 +2158,17 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>4.2 / 5.0</t>
+          <t>4.65 / 5.0 (genuine run) ; 4.2 / 5.0 (test pack)</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>Semantic phrase &amp; visual hint alignment across 10 test videos</t>
+          <t>Semantic phrase &amp; visual hint alignment</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/REPORT.md Section 4 ; timeline.json</t>
+          <t>ps3_engine/REPORT.md Section 3 ; timeline.json</t>
         </is>
       </c>
     </row>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="D9" s="24" t="inlineStr">
         <is>
-          <t>29 unit/E2E tests + 10 batch pack runs (39/39 passed)</t>
+          <t>30 unit/E2E tests + 10 batch pack runs + genuine run all passed</t>
         </is>
       </c>
       <c r="E9" s="24" t="inlineStr">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>Peak RAM: 145 MB ; GPU: 0s (CPU libx264)</t>
+          <t>Peak RAM: ~120 MB ; GPU: 0s (CPU libx264)</t>
         </is>
       </c>
       <c r="D10" s="24" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/REPORT.md Section 2.1 &amp; 4</t>
+          <t>ps3_engine/REPORT.md Section 3</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="E9" s="24" t="inlineStr">
         <is>
-          <t>ps3_engine/app/renderer.py:190-205 ; test_pack/03_coffee_promo/video_9x16.mp4</t>
+          <t>ps3_engine/app/renderer.py:190-205 ; outputs/genuine_demo_run/video_9x16.mp4</t>
         </is>
       </c>
     </row>

</xml_diff>